<commit_message>
research: Club Sizes (ON) rebuilt from the full 559-entry table — owner caught the gap
team_entries.csv (July research: NPH SL/D1 + NJC + NSC + NPA/WNPA + OSBA +
Coalition Summer 2025) is the authoritative per-club count — the md-table
parse missed the Coalition census entirely (MUMBA 18, SBA 18, YvY 12,
Toronto Lords 11). Tab renamed, double-count from the OSBA re-add avoided.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/research/provinces/SportsHub-Ontario.xlsx
+++ b/docs/research/provinces/SportsHub-Ontario.xlsx
@@ -11,14 +11,14 @@
     <sheet name="Leagues" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Club-League Map" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Contacts" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Club Sizes (ON elite)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Club Sizes (ON)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clubs'!$A$1:$P$188</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Leagues'!$A$1:$L$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Club-League Map'!$A$1:$E$264</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Contacts'!$A$1:$F$142</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Club Sizes (ON elite)'!$A$1:$D$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Club Sizes (ON)'!$A$1:$D$216</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21429,11 +21429,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D129"/>
+  <dimension ref="A1:D216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="58" customWidth="1" min="4" max="4"/>
   </cols>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Elite team entries (2025-26)</t>
+          <t>Censused team entries 2025-26</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -21466,15 +21466,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Dragons de Gatineau</t>
+          <t>Scarborough Blues / SBA (Team {coach}, Premier)</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NPH(SL + D1)=9</t>
+          <t>Coalition (Summer 2025)=18</t>
         </is>
       </c>
     </row>
@@ -21484,15 +21484,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Royal Crown</t>
+          <t>The MUMBA Mentality</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NPH(SL + D1 + NPA + WNPA)=8</t>
+          <t>Coalition (Summer 2025)=18</t>
         </is>
       </c>
     </row>
@@ -21502,15 +21502,15 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Brampton City Prep</t>
+          <t>YvY</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NJC=2; NSC=1; OSBA-coalition=5</t>
+          <t>Coalition (Summer 2025)=12</t>
         </is>
       </c>
     </row>
@@ -21520,15 +21520,15 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Wiggins Elite</t>
+          <t>Toronto Lords</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NPH(SL)=4; NJC=2; NSC=1</t>
+          <t>Coalition (Summer 2025)=7; NPH-SL=2; NSC=1; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -21538,15 +21538,15 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C.O.D.E Academy</t>
+          <t>Eurostep</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NJC=1; OSBA-coalition=6</t>
+          <t>Coalition (Summer 2025)=11</t>
         </is>
       </c>
     </row>
@@ -21556,15 +21556,15 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FEIA (Fort Erie)</t>
+          <t>Burloak</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NPH(SL + D1 + NPA + WNPA)=6</t>
+          <t>Coalition (Summer 2025)=10</t>
         </is>
       </c>
     </row>
@@ -21574,15 +21574,15 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ottawa Elite (incl. Prep)</t>
+          <t>Dragons de Gatineau</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>NPH(SL + D1)=6</t>
+          <t>NPH-SL=8; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -21592,15 +21592,15 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>St. Jude's Prep/Academy</t>
+          <t>Brampton Warriors</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NPH(D1 + NPA + WNPA)=6</t>
+          <t>Coalition (Summer 2025)=9</t>
         </is>
       </c>
     </row>
@@ -21610,15 +21610,15 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lincoln Prep</t>
+          <t>iDream by BOA</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NPH(D1 + NPA)=2; OSBA-coalition=4</t>
+          <t>Coalition (Summer 2025)=9</t>
         </is>
       </c>
     </row>
@@ -21628,15 +21628,15 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PDM Basketball</t>
+          <t>Born 2 Stand Out</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NPH(SL + D1)=5</t>
+          <t>Coalition (Summer 2025)=9</t>
         </is>
       </c>
     </row>
@@ -21646,15 +21646,15 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hodan Prep</t>
+          <t>Royal Crown</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NPH(D1 + NPA)=2; OSBA-coalition=3</t>
+          <t>NPH-SL=3; NPH-D1=3; NPA=1; WNPA=1</t>
         </is>
       </c>
     </row>
@@ -21664,15 +21664,15 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>St. Jude's Academy</t>
+          <t>Durham Blues</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>OSBA-coalition=5</t>
+          <t>Coalition (Summer 2025)=8</t>
         </is>
       </c>
     </row>
@@ -21682,15 +21682,15 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Burloak Elite</t>
+          <t>Wiggins Elite</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>NPH(SL)=4</t>
+          <t>NPH-SL=4; NJC=2; NSC=1</t>
         </is>
       </c>
     </row>
@@ -21700,15 +21700,15 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CE23 Academy</t>
+          <t>City Above</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>NPH(SL)=4</t>
+          <t>Coalition (Summer 2025)=7</t>
         </is>
       </c>
     </row>
@@ -21718,15 +21718,15 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>Hoopzone Knights</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>NPH(SL + D1)=4</t>
+          <t>Coalition (Summer 2025)=7</t>
         </is>
       </c>
     </row>
@@ -21736,15 +21736,15 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NDL</t>
+          <t>FEIA (Fort Erie)</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>NPH(D1)=4</t>
+          <t>NPH-D1=3; NPH-SL=1; NPA=1; WNPA=1</t>
         </is>
       </c>
     </row>
@@ -21754,15 +21754,15 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>North York Lions</t>
+          <t>Ottawa Elite (incl. Prep)</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>NPH(SL)=4</t>
+          <t>NPH-SL=4; NPH-D1=2</t>
         </is>
       </c>
     </row>
@@ -21772,15 +21772,15 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>RWI</t>
+          <t>St. Jude's Prep/Academy</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>NPH(SL)=4</t>
+          <t>NPH-D1=4; NPA=1; WNPA=1</t>
         </is>
       </c>
     </row>
@@ -21790,15 +21790,15 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Underdog Elite</t>
+          <t>Lincoln Prep</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>NPH(SL)=4</t>
+          <t>OSBA=4; NPH-D1=1; NPA=1</t>
         </is>
       </c>
     </row>
@@ -21808,15 +21808,15 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>City Above Elite</t>
+          <t>C.O.D.E. Academy (Provincial + International)</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NPH(SL)=3; NJC=1</t>
+          <t>OSBA=6</t>
         </is>
       </c>
     </row>
@@ -21826,15 +21826,15 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Tall Pines Academy</t>
+          <t>Future Hope Academy</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>NPH(D1)=3; OSBA-coalition=1</t>
+          <t>OSBA=3; NJC=1; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -21844,15 +21844,15 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Toronto Lords</t>
+          <t>Monarchs</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>NPH(SL + D1)=3; NSC=1</t>
+          <t>Coalition (Summer 2025)=4; NSC=1</t>
         </is>
       </c>
     </row>
@@ -21862,15 +21862,15 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ONL-X</t>
+          <t>PDM Basketball</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>NPH(SL + D1)=2; NJC=1; NSC=1</t>
+          <t>NPH-SL=4; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -21880,15 +21880,15 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Canada Topflight Academy</t>
+          <t>St. Jude's Academy (Blue + White in Trillium)</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>NJC=1; OSBA-coalition=3</t>
+          <t>OSBA=5</t>
         </is>
       </c>
     </row>
@@ -21898,15 +21898,15 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Future Hope Academy</t>
+          <t>Brampton City Prep (Nat/Prov + Reg/North + South)</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>NJC=1; OSBA-coalition=3</t>
+          <t>OSBA=5</t>
         </is>
       </c>
     </row>
@@ -21916,15 +21916,15 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Simcoe United</t>
+          <t>YNBA (incl. Avengers)</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>NJC=2; NSC=2</t>
+          <t>Coalition (Summer 2025)=5</t>
         </is>
       </c>
     </row>
@@ -21934,7 +21934,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>William Academy</t>
+          <t>City Above Elite</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -21942,7 +21942,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NJC=1; OSBA-coalition=3</t>
+          <t>NPH-SL=3; NJC=1</t>
         </is>
       </c>
     </row>
@@ -21952,7 +21952,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Royal Crown School</t>
+          <t>ONL-X</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -21960,7 +21960,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>OSBA-coalition=4</t>
+          <t>NJC=1; NSC=1; NPH-SL=1; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -21970,7 +21970,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Crestwood Prep</t>
+          <t>Simcoe United</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -21978,7 +21978,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>OSBA-coalition=4</t>
+          <t>NJC=2; NSC=2</t>
         </is>
       </c>
     </row>
@@ -21988,7 +21988,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Orangeville Prep / Athlete Institute</t>
+          <t>Burloak Elite</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -21996,7 +21996,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>OSBA-coalition=4</t>
+          <t>NPH-SL=4</t>
         </is>
       </c>
     </row>
@@ -22006,7 +22006,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Victory Academy / Victory Prep</t>
+          <t>CE23 Academy</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -22014,7 +22014,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>OSBA-coalition=4</t>
+          <t>NPH-SL=4</t>
         </is>
       </c>
     </row>
@@ -22024,15 +22024,15 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CKATT Basketball</t>
+          <t>MBA</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>NPH(SL)=3</t>
+          <t>NPH-SL=2; NPH-D1=2</t>
         </is>
       </c>
     </row>
@@ -22042,15 +22042,15 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dropoff Elite</t>
+          <t>NDL</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>NPH(SL + D1)=3</t>
+          <t>NPH-SL=3; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -22060,15 +22060,15 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Edge School (Calgary)</t>
+          <t>North York Lions</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>NPH(D1 + NPA + WNPA)=3</t>
+          <t>NPH-SL=4</t>
         </is>
       </c>
     </row>
@@ -22078,15 +22078,15 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>M and R Basketball</t>
+          <t>RWI</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>NPH(SL)=3</t>
+          <t>NPH-SL=4</t>
         </is>
       </c>
     </row>
@@ -22096,15 +22096,15 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MC Elite</t>
+          <t>Underdog Elite</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>NPH(SL)=3</t>
+          <t>NPH-SL=4</t>
         </is>
       </c>
     </row>
@@ -22114,15 +22114,15 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Polaris Prep</t>
+          <t>Tall Pines Academy</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>NPH(D1 + NPA)=3</t>
+          <t>NPH-SL=2; NPH-D1=1; OSBA=1</t>
         </is>
       </c>
     </row>
@@ -22132,15 +22132,15 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SC Academy</t>
+          <t>Royal Crown School</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>NPH(SL + D1)=3</t>
+          <t>OSBA=4</t>
         </is>
       </c>
     </row>
@@ -22150,15 +22150,15 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Simcoe United Spartans</t>
+          <t>Crestwood Prep (incl. Blue in W)</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>NPH(SL)=3</t>
+          <t>OSBA=4</t>
         </is>
       </c>
     </row>
@@ -22168,15 +22168,15 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TNP</t>
+          <t>Orangeville Prep / Athlete Institute</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>NPH(SL + D1)=3</t>
+          <t>OSBA=4</t>
         </is>
       </c>
     </row>
@@ -22186,15 +22186,15 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Tri-City (Prep/Academy)</t>
+          <t>Victory Academy / Victory Prep (East + West)</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>NPH(D1 + NPA)=3</t>
+          <t>OSBA=4</t>
         </is>
       </c>
     </row>
@@ -22204,15 +22204,15 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Vanguard North Prep</t>
+          <t>East York Eagles</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>NPH(SL)=3</t>
+          <t>Coalition (Summer 2025)=4</t>
         </is>
       </c>
     </row>
@@ -22222,7 +22222,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Westfield Secondary</t>
+          <t>Brampton City Prep</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -22230,7 +22230,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>NPH(SL + D1)=3</t>
+          <t>NJC=2; NSC=1</t>
         </is>
       </c>
     </row>
@@ -22248,7 +22248,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>NPH(SL)=2; NSC=1</t>
+          <t>NPH-SL=2; NSC=1</t>
         </is>
       </c>
     </row>
@@ -22258,7 +22258,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>G2S Game Changers</t>
+          <t>Full Circle Basketball Academy</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -22266,7 +22266,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>NPH(SL)=2; NJC=1</t>
+          <t>NJC=1; NSC=1; OSBA=1</t>
         </is>
       </c>
     </row>
@@ -22276,7 +22276,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Tru Balance</t>
+          <t>G2S Game Changers</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -22284,7 +22284,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>NPH(SL)=2; NJC=1</t>
+          <t>NPH-SL=2; NJC=1</t>
         </is>
       </c>
     </row>
@@ -22294,7 +22294,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Full Circle Basketball Academy</t>
+          <t>SC Academy Prep</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -22302,7 +22302,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>NJC=1; NSC=1; OSBA-coalition=1</t>
+          <t>NSC=2; NJC=1</t>
         </is>
       </c>
     </row>
@@ -22312,7 +22312,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SC Academy Prep</t>
+          <t>SSF Blizzard</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -22320,7 +22320,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>NJC=1; NSC=2</t>
+          <t>NJC=2; NSC=1</t>
         </is>
       </c>
     </row>
@@ -22330,7 +22330,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SSF Blizzard</t>
+          <t>Tri-City Prep</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -22338,7 +22338,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>NJC=2; NSC=1</t>
+          <t>OSBA=2; NJC=1</t>
         </is>
       </c>
     </row>
@@ -22348,7 +22348,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Tri-City Prep</t>
+          <t>Tru Balance</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -22356,7 +22356,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>NJC=1; OSBA-coalition=2</t>
+          <t>NPH-SL=2; NJC=1</t>
         </is>
       </c>
     </row>
@@ -22374,7 +22374,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>NJC=1; NSC=2</t>
+          <t>NSC=2; NJC=1</t>
         </is>
       </c>
     </row>
@@ -22384,7 +22384,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Fort Erie International Academy</t>
+          <t>CKATT Basketball</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -22392,7 +22392,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>OSBA-coalition=3</t>
+          <t>NPH-SL=3</t>
         </is>
       </c>
     </row>
@@ -22402,7 +22402,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Polaris Prep Academy</t>
+          <t>Dropoff Elite</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -22410,7 +22410,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>OSBA-coalition=3</t>
+          <t>NPH-SL=2; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -22420,7 +22420,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>King Heights Academy</t>
+          <t>Edge School (Calgary)</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -22428,7 +22428,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>OSBA-coalition=3</t>
+          <t>NPH-D1=1; NPA=1; WNPA=1</t>
         </is>
       </c>
     </row>
@@ -22438,7 +22438,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Colts Prep</t>
+          <t>M and R Basketball</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -22446,7 +22446,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>OSBA-coalition=3</t>
+          <t>NPH-SL=3</t>
         </is>
       </c>
     </row>
@@ -22456,7 +22456,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Father Henry Carr</t>
+          <t>MC Elite</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -22464,7 +22464,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>OSBA-coalition=3</t>
+          <t>NPH-SL=3</t>
         </is>
       </c>
     </row>
@@ -22474,15 +22474,15 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>BCP</t>
+          <t>Polaris Prep</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>NPH(D1 + NPA)=2</t>
+          <t>NPH-D1=2; NPA=1</t>
         </is>
       </c>
     </row>
@@ -22492,15 +22492,15 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Dynastie</t>
+          <t>SC Academy</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>NPH(D1)=2</t>
+          <t>NPH-SL=2; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -22510,15 +22510,15 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EM Elite</t>
+          <t>Simcoe United Spartans</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>NPH(SL)=2</t>
+          <t>NPH-SL=3</t>
         </is>
       </c>
     </row>
@@ -22528,15 +22528,15 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Eurostep Basketball</t>
+          <t>TNP</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>NPH(SL)=2</t>
+          <t>NPH-SL=2; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -22546,15 +22546,15 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Hamilton Transformation Academy</t>
+          <t>Tri-City (Prep/Academy)</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>NPH(SL)=2</t>
+          <t>NPH-D1=2; NPA=1</t>
         </is>
       </c>
     </row>
@@ -22564,15 +22564,15 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>King Heights</t>
+          <t>Vanguard North Prep</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>NPH(SL + NPA)=2</t>
+          <t>NPH-SL=3</t>
         </is>
       </c>
     </row>
@@ -22582,15 +22582,15 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Kings Court Basketball</t>
+          <t>Westfield Secondary</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>NPH(SL)=2</t>
+          <t>NPH-D1=2; NPH-SL=1</t>
         </is>
       </c>
     </row>
@@ -22600,15 +22600,15 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Malton Sting Basketball</t>
+          <t>Vaughan Panthers</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>NPH(SL)=2</t>
+          <t>NPH-SL=2; Coalition (Summer 2025)=1</t>
         </is>
       </c>
     </row>
@@ -22618,15 +22618,15 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>North Toronto Huskies</t>
+          <t>James Cardinal McGuigan</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>NPH(SL)=2</t>
+          <t>OSBA=2; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -22636,15 +22636,15 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Retro Elite</t>
+          <t>Niagara Prep</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>NPH(SL)=2</t>
+          <t>OSBA=2; WNPA=1</t>
         </is>
       </c>
     </row>
@@ -22654,15 +22654,15 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>St. Michael's College School</t>
+          <t>Uchenna Academy</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>NPH(SL + D1)=2</t>
+          <t>OSBA=2; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -22672,15 +22672,15 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Vaughan Panthers</t>
+          <t>Fort Erie International Academy</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>NPH(SL)=2</t>
+          <t>OSBA=3</t>
         </is>
       </c>
     </row>
@@ -22690,15 +22690,15 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Waterloo Wolverines Elite</t>
+          <t>Hodan Prep (incl. Nighthawks)</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>NPH(SL)=2</t>
+          <t>OSBA=3</t>
         </is>
       </c>
     </row>
@@ -22708,15 +22708,15 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>West United Prep</t>
+          <t>William Academy (incl. Cobourg)</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>NPH(SL)=2</t>
+          <t>OSBA=3</t>
         </is>
       </c>
     </row>
@@ -22726,15 +22726,15 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>YvY Elite</t>
+          <t>Canada Topflight Academy (Gold + Red)</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>NPH(SL)=2</t>
+          <t>OSBA=3</t>
         </is>
       </c>
     </row>
@@ -22744,15 +22744,15 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Cali Prep</t>
+          <t>Polaris Prep Academy (Gold + Black)</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>NJC=1; NSC=1</t>
+          <t>OSBA=3</t>
         </is>
       </c>
     </row>
@@ -22762,15 +22762,15 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Compass Academy</t>
+          <t>King Heights Academy</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>NJC=1; NSC=1</t>
+          <t>OSBA=3</t>
         </is>
       </c>
     </row>
@@ -22780,15 +22780,15 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>HQ Prep</t>
+          <t>Colts Prep</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>NJC=2</t>
+          <t>OSBA=3</t>
         </is>
       </c>
     </row>
@@ -22798,15 +22798,15 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Jungle Prep</t>
+          <t>Father Henry Carr (Jr. Prep + Freshmen Prep)</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>NJC=1; NSC=1</t>
+          <t>OSBA=3</t>
         </is>
       </c>
     </row>
@@ -22816,7 +22816,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>Alpha Elite</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -22824,7 +22824,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>NJC=1; NSC=1</t>
+          <t>NJC=1; NPH-SL=1</t>
         </is>
       </c>
     </row>
@@ -22834,7 +22834,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>London Ramblers</t>
+          <t>Cali Prep</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -22842,7 +22842,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>NJC=2</t>
+          <t>NJC=1; NSC=1</t>
         </is>
       </c>
     </row>
@@ -22852,7 +22852,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Project Excellence</t>
+          <t>Compass Academy</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -22870,7 +22870,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SBA Premier</t>
+          <t>Eastern Basketball Academy</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -22878,7 +22878,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>NJC=1; NSC=1</t>
+          <t>NJC=1; NPH-SL=1</t>
         </is>
       </c>
     </row>
@@ -22888,7 +22888,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Top Notch Prep</t>
+          <t>HQ Prep</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -22906,7 +22906,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Westfield Prep</t>
+          <t>Jungle Prep</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -22924,7 +22924,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Wolverines Elite</t>
+          <t>LBA</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -22942,7 +22942,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Inspire Academy</t>
+          <t>London Ramblers</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -22950,7 +22950,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>OSBA-coalition=2</t>
+          <t>NJC=2</t>
         </is>
       </c>
     </row>
@@ -22960,7 +22960,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Lo-Ellen Park Prep</t>
+          <t>Orangeville Prep</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -22968,7 +22968,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>OSBA-coalition=2</t>
+          <t>NSC=1; NPH-SL=1</t>
         </is>
       </c>
     </row>
@@ -22978,7 +22978,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Niagara Prep</t>
+          <t>Project Excellence</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -22986,7 +22986,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>OSBA-coalition=2</t>
+          <t>NJC=1; NSC=1</t>
         </is>
       </c>
     </row>
@@ -22996,7 +22996,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>J.Addison School</t>
+          <t>SBA Premier</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -23004,7 +23004,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>OSBA-coalition=2</t>
+          <t>NJC=1; NSC=1</t>
         </is>
       </c>
     </row>
@@ -23014,7 +23014,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Capital Courts Academy</t>
+          <t>Ste Cecile Academy</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -23022,7 +23022,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>OSBA-coalition=2</t>
+          <t>NSC=1; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -23032,7 +23032,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Louis-Riel</t>
+          <t>Top Notch Prep</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -23040,7 +23040,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>OSBA-coalition=2</t>
+          <t>NJC=2</t>
         </is>
       </c>
     </row>
@@ -23050,7 +23050,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>H5 Academy</t>
+          <t>Westfield Prep</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -23058,7 +23058,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>OSBA-coalition=2</t>
+          <t>NJC=1; NSC=1</t>
         </is>
       </c>
     </row>
@@ -23068,7 +23068,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>James Cardinal McGuigan</t>
+          <t>Wolverines Elite</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -23076,7 +23076,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>OSBA-coalition=2</t>
+          <t>NJC=1; NSC=1</t>
         </is>
       </c>
     </row>
@@ -23086,7 +23086,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Uchenna Academy</t>
+          <t>BCP</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -23094,7 +23094,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>OSBA-coalition=2</t>
+          <t>NPH-D1=1; NPA=1</t>
         </is>
       </c>
     </row>
@@ -23104,15 +23104,15 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>506 Elite Jr Academy</t>
+          <t>Dynastie</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>NPH-D1=2</t>
         </is>
       </c>
     </row>
@@ -23122,15 +23122,15 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Against The Six Prep</t>
+          <t>EM Elite</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>NPH-SL=2</t>
         </is>
       </c>
     </row>
@@ -23140,15 +23140,15 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Alpha Elite</t>
+          <t>Eurostep Basketball</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>NPH-SL=2</t>
         </is>
       </c>
     </row>
@@ -23158,15 +23158,15 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>CKATT</t>
+          <t>Hamilton Transformation Academy</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>NPH-SL=2</t>
         </is>
       </c>
     </row>
@@ -23176,15 +23176,15 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Collective Elite Academy</t>
+          <t>Hodan Prep</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>NPH-D1=1; NPA=1</t>
         </is>
       </c>
     </row>
@@ -23194,15 +23194,15 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Cooksville We&gt;Me</t>
+          <t>King Heights</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>NPH-SL=1; NPA=1</t>
         </is>
       </c>
     </row>
@@ -23212,15 +23212,15 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Dynamic Basketball</t>
+          <t>Kings Court Basketball</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>NSC=1</t>
+          <t>NPH-SL=2</t>
         </is>
       </c>
     </row>
@@ -23230,15 +23230,15 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Eastern Basketball Academy</t>
+          <t>Malton Sting Basketball</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>NPH-SL=2</t>
         </is>
       </c>
     </row>
@@ -23248,15 +23248,15 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Elton Academy</t>
+          <t>North Toronto Huskies</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>NSC=1</t>
+          <t>NPH-SL=2</t>
         </is>
       </c>
     </row>
@@ -23266,15 +23266,15 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>F.O.R.M. Basketball Academy</t>
+          <t>Retro Elite</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>NSC=1</t>
+          <t>NPH-SL=2</t>
         </is>
       </c>
     </row>
@@ -23284,15 +23284,15 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Gators Basketball Academy</t>
+          <t>St. Michael's College School</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>NSC=1</t>
+          <t>NPH-SL=1; NPH-D1=1</t>
         </is>
       </c>
     </row>
@@ -23302,15 +23302,15 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>GBU</t>
+          <t>Waterloo Wolverines Elite</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>NSC=1</t>
+          <t>NPH-SL=2</t>
         </is>
       </c>
     </row>
@@ -23320,15 +23320,15 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Ignite Academy</t>
+          <t>West United Prep</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>NPH-SL=2</t>
         </is>
       </c>
     </row>
@@ -23338,15 +23338,15 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Kings Court Academy</t>
+          <t>YvY Elite</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>NPH-SL=2</t>
         </is>
       </c>
     </row>
@@ -23356,15 +23356,15 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>M&amp;R Basketball</t>
+          <t>King's Christian Collegiate</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>NSC=1</t>
+          <t>WNPA=1; OSBA=1</t>
         </is>
       </c>
     </row>
@@ -23374,15 +23374,15 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Monarchs</t>
+          <t>Ridley College</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>NSC=1</t>
+          <t>NPA=1; OSBA=1</t>
         </is>
       </c>
     </row>
@@ -23392,15 +23392,15 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>NSE Select Academy</t>
+          <t>Southwest Academy</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>NPH-D1=1; OSBA=1</t>
         </is>
       </c>
     </row>
@@ -23410,15 +23410,15 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Orangeville Prep</t>
+          <t>Inspire Academy</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>NSC=1</t>
+          <t>OSBA=2</t>
         </is>
       </c>
     </row>
@@ -23428,15 +23428,15 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>RSB Elite</t>
+          <t>Lo-Ellen Park Prep</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>OSBA=2</t>
         </is>
       </c>
     </row>
@@ -23446,15 +23446,15 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>RWI519</t>
+          <t>J.Addison School</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>OSBA=2</t>
         </is>
       </c>
     </row>
@@ -23464,15 +23464,15 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>SCI Spartans</t>
+          <t>Capital Courts Academy</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>OSBA=2</t>
         </is>
       </c>
     </row>
@@ -23482,15 +23482,15 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Ste Cecile Academy</t>
+          <t>Louis-Riel (Academy)</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>NSC=1</t>
+          <t>OSBA=2</t>
         </is>
       </c>
     </row>
@@ -23500,15 +23500,15 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Strive Hoops</t>
+          <t>H5 Academy</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>OSBA=2</t>
         </is>
       </c>
     </row>
@@ -23518,15 +23518,15 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Team Sanctuary</t>
+          <t>Durham Rising Suns</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>Coalition (Summer 2025)=2</t>
         </is>
       </c>
     </row>
@@ -23536,15 +23536,15 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Team Thetford</t>
+          <t>K-W Vipers</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>NSC=1</t>
+          <t>Coalition (Summer 2025)=2</t>
         </is>
       </c>
     </row>
@@ -23554,15 +23554,15 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Top Left</t>
+          <t>Milton Stags</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>NJC=1</t>
+          <t>Coalition (Summer 2025)=2</t>
         </is>
       </c>
     </row>
@@ -23572,7 +23572,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Triple Balance</t>
+          <t>506 Elite Jr Academy</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -23580,7 +23580,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>NSC=1</t>
+          <t>NJC=1</t>
         </is>
       </c>
     </row>
@@ -23590,7 +23590,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>UEWB</t>
+          <t>Against The Six Prep</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -23608,7 +23608,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Ridley College</t>
+          <t>C.O.D.E Academy</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -23616,7 +23616,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>OSBA-coalition=1</t>
+          <t>NJC=1</t>
         </is>
       </c>
     </row>
@@ -23626,7 +23626,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Cambridge International Academy</t>
+          <t>Canada Topflight Academy</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -23634,7 +23634,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>OSBA-coalition=1</t>
+          <t>NJC=1</t>
         </is>
       </c>
     </row>
@@ -23644,7 +23644,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>King's Christian Collegiate</t>
+          <t>CKATT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -23652,7 +23652,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>OSBA-coalition=1</t>
+          <t>NJC=1</t>
         </is>
       </c>
     </row>
@@ -23662,7 +23662,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Redmond Basketball</t>
+          <t>Collective Elite Academy</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -23670,7 +23670,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>OSBA-coalition=1</t>
+          <t>NJC=1</t>
         </is>
       </c>
     </row>
@@ -23680,7 +23680,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Richmond Hill Ascend Prep</t>
+          <t>Cooksville We&gt;Me</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -23688,7 +23688,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>OSBA-coalition=1</t>
+          <t>NJC=1</t>
         </is>
       </c>
     </row>
@@ -23698,7 +23698,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Ace Acumen Heights</t>
+          <t>Dynamic Basketball</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -23706,7 +23706,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>OSBA-coalition=1</t>
+          <t>NSC=1</t>
         </is>
       </c>
     </row>
@@ -23716,7 +23716,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>AD Rebelles</t>
+          <t>Elton Academy</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -23724,7 +23724,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>OSBA-coalition=1</t>
+          <t>NSC=1</t>
         </is>
       </c>
     </row>
@@ -23734,7 +23734,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Southwest Academy</t>
+          <t>F.O.R.M. Basketball Academy</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -23742,7 +23742,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>OSBA-coalition=1</t>
+          <t>NSC=1</t>
         </is>
       </c>
     </row>
@@ -23752,7 +23752,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>St. Michael's College</t>
+          <t>Gators Basketball Academy</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -23760,12 +23760,1578 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>OSBA-coalition=1</t>
+          <t>NSC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>GBU</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>1</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>NSC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Ignite Academy</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>1</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>NJC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Kings Court Academy</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>1</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>NJC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>M&amp;R Basketball</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>1</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>NSC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>NSE Select Academy</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>1</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>NJC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>RSB Elite</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>1</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>NJC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>RWI519</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>1</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>NJC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>SCI Spartans</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>1</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>NJC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Strive Hoops</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>1</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>NJC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Team Sanctuary</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>1</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>NJC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Team Thetford</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>1</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>NSC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Top Left</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>1</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>NJC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Triple Balance</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>NSC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>UEWB</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>1</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>NJC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>William Academy</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>1</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>NJC=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>AAA Academy</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>1</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Against the Six</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>1</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Alma Prep</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>1</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>B1CE London</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>1</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>BALL905 Elite</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>1</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Barrie Buccaneers</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>1</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Blessed Sacrament</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>1</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Brantford Hawks</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Burlington Force</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>1</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Burlington Hoops Academy</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>1</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>C.O.D.E Sports Academy</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>1</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>WNPA=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>CB Elite</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>1</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>CSJV Prep Basketball QC</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>1</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>NPA=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Canada Central Prep</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>1</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Canadian Private School</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>1</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Capital Courts</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>1</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Cathedral</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>1</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Crestwood Prep</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>1</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>NPA=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>DEl1te</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>1</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>DFA Academy</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>1</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Dundas Dynamo</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>1</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Durham Gators</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>1</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>École St-Gabriel Escadron</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>1</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Father Henry Carr</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>1</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>First Step Elite Gold</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>1</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Fitz Youth</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>1</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Fundamentals First</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>GT Elite</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>1</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>GYBA Gryphons</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>1</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Grassroots Niagara</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>1</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Gwillimbury Basketball United</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>1</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>HQ Elite</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>1</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Hamilton Elite</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>1</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>HoopHer</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>1</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Hooptrotters OGs</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>1</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>J. Addison Jaguars</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>1</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>K9 Elite White</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>1</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Lead2Greatness</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>1</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Mississauga Monarchs</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>1</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Momentum Basketball</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>1</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Norwood Stars</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>1</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Notre Dame Hounds SK</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>1</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>WNPA=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Oakville Panthers</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>1</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Oakville Vytis</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>1</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Orillia Lakers</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>1</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Ottawa Prospects</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>1</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Prolific Sports Academy</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>1</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Rothesay Netherwood School NB</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>1</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>NPA=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Sacred Heart Montreal</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>1</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>WNPA=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>TC Soldiers</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>1</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Team CB</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>1</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>The Conglomerate</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>1</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Thornhill Thunder</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>1</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Tornades Basketball</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>1</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Toronto Top Tier East</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>1</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Union Elite</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>1</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Victory Prep</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>1</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>West Ottawa</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>1</v>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>William Prep</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>1</v>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>NPH-D1=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>YASO Basketball Academy Black</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>1</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>NPH-SL=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Cambridge International Academy</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>1</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>OSBA=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Redmond Basketball</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>1</v>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>OSBA=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Richmond Hill Ascend Prep</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>1</v>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>OSBA=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Ace Acumen Heights</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>1</v>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>OSBA=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>AD Rebelles</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>1</v>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>OSBA=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>St. Michael's College</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>1</v>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>OSBA=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>210</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>North Toronto Huskies (NTBA)</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>1</v>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Coalition (Summer 2025)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>211</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Etobicoke Thunder</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>1</v>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Coalition (Summer 2025)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Barrie Royals</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>1</v>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Coalition (Summer 2025)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Blessed Sacrament (Yellow Jackets)</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>1</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Coalition (Summer 2025)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Toronto Triple Threat</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>1</v>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Coalition (Summer 2025)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Silver Knights (SilverKnights Elite)</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>1</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Coalition (Summer 2025)=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D129"/>
+  <autoFilter ref="A1:D216"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>